<commit_message>
fix(import)!: P0 never link a child to an existing parent account with a different name (PHONE_NAME_MISMATCH row error, 422 on import; same phone/different names within the file too; NFC + case/whitespace-insensitive, diacritics kept); explicit override via multipart confirmLinks; DELETE /children/:id/guardians/:guardianId (admin, reason required, audit.jsonl); tests with tester P0 files
</commit_message>
<xml_diff>
--- a/deploy/templates/mau-nhap-hoc-sinh.xlsx
+++ b/deploy/templates/mau-nhap-hoc-sinh.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Họ tên bé *</t>
   </si>
@@ -218,6 +218,12 @@
   </si>
   <si>
     <t>SĐT chưa có tài khoản → tạo tài khoản phụ huynh, mật khẩu tạm có trong file kết quả (chỉ tải được một lần), bắt đổi khi đăng nhập lần đầu. SĐT đã có tài khoản phụ huynh → gắn bé vào tài khoản đó.</t>
+  </si>
+  <si>
+    <t>SĐT đã có tài khoản</t>
+  </si>
+  <si>
+    <t>SĐT đã là tài khoản phụ huynh nhưng khác tên (không phân biệt hoa thường / khoảng trắng; CÓ phân biệt dấu) → LỖI, không gắn. Cùng một SĐT ghi tên khác nhau ở các dòng → LỖI. Nếu nhà trường đã xác minh đúng là cùng một người: xác nhận gắn trên màn hình nhập (từng dòng, từng phụ huynh).</t>
   </si>
   <si>
     <t>Trùng</t>
@@ -4783,7 +4789,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -4870,6 +4876,14 @@
         <v>35</v>
       </c>
     </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>